<commit_message>
add more ER and BA graphs
</commit_message>
<xml_diff>
--- a/randoms_BA/randoms_BA_annotations_scores_wo_lgl.xlsx
+++ b/randoms_BA/randoms_BA_annotations_scores_wo_lgl.xlsx
@@ -394,7 +394,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -663,6 +663,259 @@
         <v>1</v>
       </c>
     </row>
+    <row r="12" spans="1:7">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>6</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>4</v>
+      </c>
+      <c r="F12">
+        <v>5</v>
+      </c>
+      <c r="G12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>6</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13">
+        <v>5</v>
+      </c>
+      <c r="E13">
+        <v>4</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <v>6</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>5</v>
+      </c>
+      <c r="E14">
+        <v>4</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15">
+        <v>6</v>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
+      <c r="D15">
+        <v>5</v>
+      </c>
+      <c r="E15">
+        <v>2</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>6</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>2</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>5</v>
+      </c>
+      <c r="G16">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>6</v>
+      </c>
+      <c r="C17">
+        <v>5</v>
+      </c>
+      <c r="D17">
+        <v>4</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>6</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>4</v>
+      </c>
+      <c r="E18">
+        <v>5</v>
+      </c>
+      <c r="F18">
+        <v>2</v>
+      </c>
+      <c r="G18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19">
+        <v>6</v>
+      </c>
+      <c r="C19">
+        <v>4</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <v>3</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <v>6</v>
+      </c>
+      <c r="C20">
+        <v>2</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>3</v>
+      </c>
+      <c r="F20">
+        <v>5</v>
+      </c>
+      <c r="G20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21">
+        <v>19</v>
+      </c>
+      <c r="B21">
+        <v>6</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>3</v>
+      </c>
+      <c r="F21">
+        <v>5</v>
+      </c>
+      <c r="G21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22">
+        <v>5</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
+        <v>6</v>
+      </c>
+      <c r="E22">
+        <v>2</v>
+      </c>
+      <c r="F22">
+        <v>4</v>
+      </c>
+      <c r="G22">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>